<commit_message>
Read chartsheets, fix BOM-prefixed part offsets, and refuse newer error values with a typed code
- Python and Rust list chartsheets (name -> part) and preserve them byte-for-byte instead of
  refusing the workbook; localSheetId now counts every sheet entry, chartsheets included.
  Dialog and macro sheets still refuse, now as unsupported_sheet_type.
- Rust: quick-xml positions start after a UTF-8 byte-order mark; offsets are shifted so
  patches splice into the original bytes (BOM-prefixed worksheets exported invalid XML).
- Stored error values outside the v1 error set (#GETTING_DATA, #FIELD!, #BLOCKED!, ...)
  refuse as unsupported_error_value in both engines; the model's error enum is unchanged.
  The corpus splits hb_errors_as_values (v1 set) from hb_errors_newer_values.
- generate_corpus.py --writers regenerates one writer's files without touching the others.
</commit_message>
<xml_diff>
--- a/fixtures/corpus/hb_errors_as_values.xlsx
+++ b/fixtures/corpus/hb_errors_as_values.xlsx
@@ -43,7 +43,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="e">
@@ -119,18 +119,10 @@
     </row>
     <row r="10">
       <c r="A10" t="e">
-        <v>#GETTING_DATA</v>
-      </c>
-      <c r="B10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="e">
         <f>1/0</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="B11" t="b">
+      <c r="B10" t="b">
         <f>B1</f>
         <v>1</v>
       </c>

</xml_diff>